<commit_message>
Export als CSV Button entfernt
</commit_message>
<xml_diff>
--- a/Output/Win64/Release/Dokumente/Inventarliste.xlsx
+++ b/Output/Win64/Release/Dokumente/Inventarliste.xlsx
@@ -7,10 +7,10 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="21359" windowHeight="8174"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="flId1"/>
+    <sheet name="Inventar" sheetId="1" r:id="flId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" hidden="1" localSheetId="0">Sheet1!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" hidden="1" localSheetId="0">Inventar!$A$1:$J$1</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -3929,7 +3929,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4122,8 +4122,14 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -4253,6 +4259,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="61">
     <xf fontId="0" numFmtId="0" fillId="0" borderId="0"/>
@@ -4317,8 +4332,9 @@
     <xf applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0" fontId="19" numFmtId="0" fillId="0" borderId="9"/>
     <xf applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0" fontId="17" numFmtId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf fontId="0" numFmtId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf applyFont="1" applyFill="1" applyBorder="1" fontId="19" numFmtId="0" fillId="33" borderId="11" xfId="0"/>
   </cellXfs>
   <cellStyles count="61">
     <cellStyle name="20% - Accent1" xfId="15" builtinId="30"/>
@@ -4691,34 +4707,34 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>